<commit_message>
Adding separate folder for research figures
</commit_message>
<xml_diff>
--- a/analysis/correlation_summary_table.xlsx
+++ b/analysis/correlation_summary_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e04d2cc7e59c36d5/Documents/Python/MUSHRA/analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="11_2B5906BF17D1D2106487F633533088B35299F049" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84448938-8142-4095-A40A-5E41CD4733B1}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_2B5906BF17D1D2106487F633533088B35299F049" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3432B56-7AB8-4EB0-9414-8A7A4F4CAB25}"/>
   <bookViews>
     <workbookView xWindow="2928" yWindow="2928" windowWidth="17280" windowHeight="10680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -198,7 +198,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -213,17 +213,121 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="8">
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -259,123 +363,6 @@
         </horizontal>
       </border>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="15" formatCode="0.00E+00"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -394,22 +381,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>510540</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>7620</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>281940</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+        <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3635BFEA-F483-150B-4C79-C8DB89E206D4}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3C048371-01C4-6BD0-2168-160B15CB34F6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -432,7 +419,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="4030980" y="1828800"/>
+          <a:off x="4541520" y="1333500"/>
           <a:ext cx="3429000" cy="1104900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -460,7 +447,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E90DD6BF-C043-44DE-83F5-A3D761298003}" name="Table1" displayName="Table1" ref="A1:D6" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E90DD6BF-C043-44DE-83F5-A3D761298003}" name="Table1" displayName="Table1" ref="A1:D6" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="6" tableBorderDxfId="5" totalsRowBorderDxfId="4">
   <autoFilter ref="A1:D6" xr:uid="{E90DD6BF-C043-44DE-83F5-A3D761298003}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -468,10 +455,10 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{059D13E7-3C50-4D27-B026-D0D6CD357B7E}" name="Comparison" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{A3CCDCD4-9B28-4FC0-970D-643F769EC0A4}" name="n" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{B8D916F7-EFD5-4CDC-B342-7DB8304CD6C3}" name="Spearman ρ" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{BEB90397-9758-4EDF-A5CF-EFFCF2025C86}" name="p-value" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{059D13E7-3C50-4D27-B026-D0D6CD357B7E}" name="Comparison" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{A3CCDCD4-9B28-4FC0-970D-643F769EC0A4}" name="n" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{B8D916F7-EFD5-4CDC-B342-7DB8304CD6C3}" name="Spearman ρ" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{BEB90397-9758-4EDF-A5CF-EFFCF2025C86}" name="p-value" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -796,7 +783,7 @@
       <c r="C2" s="7">
         <v>1</v>
       </c>
-      <c r="D2" s="8">
+      <c r="D2" s="11">
         <v>0</v>
       </c>
     </row>
@@ -810,7 +797,7 @@
       <c r="C3" s="7">
         <v>-1</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="11">
         <v>0</v>
       </c>
     </row>
@@ -824,7 +811,7 @@
       <c r="C4" s="7">
         <v>-0.5</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="11">
         <v>0.66669999999999996</v>
       </c>
     </row>
@@ -838,21 +825,21 @@
       <c r="C5" s="7">
         <v>-1</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="11">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="9">
         <v>3</v>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="10">
         <v>-0.5</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="12">
         <v>0.66669999999999996</v>
       </c>
     </row>

</xml_diff>